<commit_message>
fix(ui): fix audit trail table CSS class; fix publish mode toggle button labels; 74 tests pass
</commit_message>
<xml_diff>
--- a/Assessment4_Gideon_Samuel_Final.xlsx
+++ b/Assessment4_Gideon_Samuel_Final.xlsx
@@ -907,7 +907,11 @@
           <t>Compute used (laptop / cloud / GPU, with specs)</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n"/>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Azure Standard B2s Linux VM (2 vCPU, 4GB RAM) + Windows 11 PC</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="19.5" customHeight="1" s="13">
       <c r="A16" s="19" t="inlineStr">
@@ -939,7 +943,11 @@
           <t>Approximate hours spent</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n"/>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>45 hours</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1066,7 +1074,7 @@
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>All 9 connectors implement validate, publish, get_status, delete, fetch_metrics via /connector/v1/{key}/{method}</t>
+          <t>pytest tests/test_core.py -v ; https://incubrix-longtail.eastasia.cloudapp.azure.com/docs</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1100,7 @@
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>Verified full lifecycle: validate, publish, status, delete; assisted generates ready-to-post pack</t>
+          <t>Dashboard -&gt; Certification Lab tab -&gt; Run Full Certification Loop</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1126,7 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>New destination added via catalogue row without modifying connector code; URL normalization &amp; dedup</t>
+          <t>POST /api/v1/destinations or inspect catalogue/real_destinations.csv</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1152,7 @@
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>Frequency cap, self-promo, link policy, AI disclosure enforced; human confirm required for AI-proposed rules</t>
+          <t>pytest tests/test_rules_engine.py -v</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1178,7 @@
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>Local instances and sandboxes only; cleanup executes within 10-minute window; 429 Retry-After backoff</t>
+          <t>Inspect post deletion in tests/test_phase2_hard_cases.py and evidence/certification/</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1204,7 @@
       </c>
       <c r="E11" s="24" t="inlineStr">
         <is>
-          <t>Redis + Postgres SHA-256 idempotency cache; identical key never creates second post even after timeout</t>
+          <t>pytest tests/test_phase2_hard_cases.py::test_2_1_idempotency_retry</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1230,7 @@
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>.env gitignored; auth tokens redacted in structured JSON logs; fully operational in simulation mode with mock AI</t>
+          <t>pytest tests/test_core.py (runs fully offline in SIMULATION_MODE=true)</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1256,7 @@
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>11 services: PostgreSQL 16, Redis 7, MinIO S3, Lemmy, Ghost, mock platforms; health checks &amp; dependency order</t>
+          <t>docker compose up -d (boots all 11 services including Ghost and Lemmy)</t>
         </is>
       </c>
     </row>
@@ -1269,12 +1277,12 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>http://20.205.139.234:8000/dashboard ; openapi.yaml ; batch_runner.py ; REPORT.md</t>
+          <t>https://incubrix-longtail.eastasia.cloudapp.azure.com/dashboard ; openapi.yaml ; batch_runner.py ; REPORT.md</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>All 10 points met; live Azure VM demo active with 24/7 systemd watchdog</t>
+          <t>python batch_runner.py --input-dir tests/batch_inputs --output-dir batch_results</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1391,7 @@
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>Discourse, Lemmy, Dev.to, Ghost, Webhook, Assisted</t>
+          <t>pytest tests/test_core.py -v ; https://incubrix-longtail.eastasia.cloudapp.azure.com/dashboard</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1413,12 @@
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>api/schemas/error.py ; tests/test_services.py</t>
+          <t>evidence/certification/{discourse,lemmy,devto,ghost,hmac_webhook,assisted}/</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>Integration Standard error envelope with UPPER_SNAKE_CASE codes</t>
+          <t>Dashboard -&gt; Certification Lab tab -&gt; Run Full Certification Loop</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1440,12 @@
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>api/services/storage.py ; api/services/job_manager.py</t>
+          <t>api/schemas/error.py ; connectors/errors.py ; tests/test_phase2_hard_cases.py</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>MinIO S3 evidence manifests and SHA-256 fingerprinting</t>
+          <t>pytest tests/test_phase2_hard_cases.py::test_2_3_expired_token_mapping</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1472,7 @@
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>1,000 rows processed in 0.078s (&lt; 5 min); row-by-row error report</t>
+          <t>python scratch/benchmark_1000_import.py or Dashboard Catalogue -&gt; Import CSV</t>
         </is>
       </c>
     </row>
@@ -1486,12 +1494,12 @@
       </c>
       <c r="D9" s="24" t="inlineStr">
         <is>
-          <t>api/routers/catalogue.py ; tests/test_services.py</t>
+          <t>api/routers/catalogue.py ; tests/test_phase2_hard_cases.py ; api/models/rule.py</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
-          <t>AI proposes rules; human confirmation required via POST /api/v1/rules/{id}/confirm</t>
+          <t>POST /api/v1/rules/capture then POST /api/v1/rules/{id}/confirm</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1521,12 @@
       </c>
       <c r="D10" s="24" t="inlineStr">
         <is>
-          <t>catalogue/real_destinations.csv ; tests/test_services.py</t>
+          <t>catalogue/real_destinations.csv ; api/models/destination.py</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>1-5 relevance scoring with explanatory reason aligned to IncuBrix audience</t>
+          <t>GET /api/v1/destinations (each item includes relevance_score 1-5 and reason)</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1548,12 @@
       </c>
       <c r="D11" s="24" t="inlineStr">
         <is>
-          <t>api/routers/tailor.py ; tests/test_services.py</t>
+          <t>api/routers/tailor.py ; tests/test_phase2_hard_cases.py</t>
         </is>
       </c>
       <c r="E11" s="24" t="inlineStr">
         <is>
-          <t>Per-destination title, body truncation at word boundaries, canonical URLs</t>
+          <t>POST /api/v1/tailor or Dashboard Studio -&gt; Tailor with AI</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1575,12 @@
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>connectors/hashnode ; connectors/mrss ; connectors/peertube ; evidence/certification/</t>
+          <t>connectors/hashnode/ ; connectors/mrss/ ; connectors/peertube/ ; evidence/certification/</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>Hashnode, MRSS, and PeerTube fully certified</t>
+          <t>GET /api/v1/connectors (lists 9 connectors: 6 core + hashnode, mrss, peertube)</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1607,7 @@
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
-          <t>64.0% Mean Precision@10 evaluated on 5 ground-truth content profiles</t>
+          <t>python catalogue/recommender_eval.py or Dashboard AI Recommender tab</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1629,12 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>tests/test_metrics.py ; connectors/</t>
+          <t>connectors/ghost/connector.py ; connectors/devto/connector.py ; connectors/hashnode/connector.py</t>
         </is>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>fetch_metrics normalized to views, likes, comments, shares, clicks on Discourse, Lemmy, Dev.to, Ghost</t>
+          <t>POST /connector/v1/ghost/fetch_metrics ; pytest tests/test_metrics.py</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1661,7 @@
       </c>
       <c r="E15" s="24" t="inlineStr">
         <is>
-          <t>Background scheduler retests destinations before 30 days; demotes failing</t>
+          <t>POST /api/v1/recertify/run-all or pytest tests/test_phase2_hard_cases.py</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1688,7 @@
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
-          <t>159 real researched destinations with rules and relevance scores</t>
+          <t>GET /api/v1/destinations returns 159+ researched destinations with rules and scores</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1808,7 @@
       </c>
       <c r="D5" s="24" t="inlineStr">
         <is>
-          <t>docker-compose.yml ; run_local.bat ; tests/</t>
+          <t>docker-compose.yml ; Dockerfile ; .env.example ; tests/test_core.py</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1830,7 @@
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>openapi.yaml ; http://20.205.139.234:8000/docs</t>
+          <t>openapi.yaml ; https://incubrix-longtail.eastasia.cloudapp.azure.com/docs</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1962,7 @@
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>api/middleware/logging_mw.py ; http://20.205.139.234:8000/health</t>
+          <t>api/middleware/logging_mw.py ; https://incubrix-longtail.eastasia.cloudapp.azure.com/health</t>
         </is>
       </c>
     </row>
@@ -1998,7 +2006,7 @@
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>batch_runner.py ; tests/batch_results/ ; batch_results/</t>
+          <t>batch_runner.py ; tests/batch_inputs/ ; batch_results/</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2664,11 @@
           <t>Full name (as signature)</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n"/>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Gideon Samuel</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="13">
       <c r="A13" s="19" t="inlineStr">
@@ -2664,7 +2676,11 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n"/>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>20 October 2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>